<commit_message>
update case of residential crime study
</commit_message>
<xml_diff>
--- a/Case of residential crime study/Case of residential crime study.xlsx
+++ b/Case of residential crime study/Case of residential crime study.xlsx
@@ -391,10 +391,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.1929012345679012</v>
+        <v>0.07439999999999999</v>
       </c>
       <c r="D2">
-        <v>5.474672474409928E-05</v>
+        <v>7.804437058098957E-28</v>
       </c>
     </row>
     <row r="3">
@@ -409,10 +409,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.2469135802469136</v>
+        <v>0.1336</v>
       </c>
       <c r="D3">
-        <v>0.004864208186179272</v>
+        <v>8.589914961212566E-12</v>
       </c>
     </row>
     <row r="4">
@@ -427,10 +427,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.1095679012345679</v>
+        <v>0.0472</v>
       </c>
       <c r="D4">
-        <v>3.08794865172942E-10</v>
+        <v>1.512896130081941E-42</v>
       </c>
     </row>
     <row r="5">
@@ -445,10 +445,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.1234567901234568</v>
+        <v>0.0464</v>
       </c>
       <c r="D5">
-        <v>4.804442753242007E-09</v>
+        <v>1.582279896822512E-44</v>
       </c>
     </row>
     <row r="6">
@@ -463,10 +463,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.1728395061728395</v>
+        <v>0.0696</v>
       </c>
       <c r="D6">
-        <v>7.587769234624996E-06</v>
+        <v>1.250759598003088E-29</v>
       </c>
     </row>
     <row r="7">
@@ -481,10 +481,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.2561728395061729</v>
+        <v>0.1152</v>
       </c>
       <c r="D7">
-        <v>0.007722215987824777</v>
+        <v>9.128475680692894E-15</v>
       </c>
     </row>
   </sheetData>
@@ -531,10 +531,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.2372003598376317</v>
+        <v>0.2409946417943775</v>
       </c>
       <c r="D2">
-        <v>0.1007863699619085</v>
+        <v>0.09529596052654821</v>
       </c>
     </row>
     <row r="3">
@@ -549,10 +549,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.6419288059776628</v>
+        <v>0.5758561426755622</v>
       </c>
       <c r="D3">
-        <v>6.657865290193854E-07</v>
+        <v>1.496551076263231E-05</v>
       </c>
     </row>
     <row r="4">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.4077414146794142</v>
+        <v>0.4016465624792653</v>
       </c>
       <c r="D4">
-        <v>0.003636923169701767</v>
+        <v>0.004230060809255809</v>
       </c>
     </row>
     <row r="5">
@@ -585,10 +585,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.6018242990998784</v>
+        <v>0.5611671771902005</v>
       </c>
       <c r="D5">
-        <v>4.78484692201242E-06</v>
+        <v>2.735352199456642E-05</v>
       </c>
     </row>
     <row r="6">
@@ -603,10 +603,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.1981525002572533</v>
+        <v>0.2264557778720811</v>
       </c>
       <c r="D6">
-        <v>0.1723041877953277</v>
+        <v>0.1176598148571866</v>
       </c>
     </row>
     <row r="7">
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.3556509555148407</v>
+        <v>0.3630723600274959</v>
       </c>
       <c r="D7">
-        <v>0.01214582219349691</v>
+        <v>0.01034582954412855</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
re-execute case study 1
</commit_message>
<xml_diff>
--- a/Case of residential crime study/Case of residential crime study.xlsx
+++ b/Case of residential crime study/Case of residential crime study.xlsx
@@ -10,7 +10,8 @@
     <sheet name="gcmc" sheetId="1" r:id="rId1"/>
     <sheet name="gccm" sheetId="2" r:id="rId2"/>
     <sheet name="pcc" sheetId="3" r:id="rId3"/>
-    <sheet name="gd" sheetId="4" r:id="rId4"/>
+    <sheet name="directlingam" sheetId="4" r:id="rId4"/>
+    <sheet name="gd" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -391,10 +392,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.0808</v>
+        <v>0.1634349030470914</v>
       </c>
       <c r="D2">
-        <v>8.072164768242996E-23</v>
+        <v>1.113718253058543E-06</v>
       </c>
     </row>
     <row r="3">
@@ -409,10 +410,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.1432</v>
+        <v>0.2770083102493075</v>
       </c>
       <c r="D3">
-        <v>1.022037555902064E-10</v>
+        <v>0.01527903552419327</v>
       </c>
     </row>
     <row r="4">
@@ -427,10 +428,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.0472</v>
+        <v>0.09279778393351801</v>
       </c>
       <c r="D4">
-        <v>1.512896130081941E-42</v>
+        <v>6.863120703650568E-14</v>
       </c>
     </row>
     <row r="5">
@@ -445,10 +446,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.0496</v>
+        <v>0.0997229916897507</v>
       </c>
       <c r="D5">
-        <v>7.690666776785052E-43</v>
+        <v>5.228570704122775E-12</v>
       </c>
     </row>
     <row r="6">
@@ -463,10 +464,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.076</v>
+        <v>0.1578947368421053</v>
       </c>
       <c r="D6">
-        <v>6.514867964944103E-24</v>
+        <v>5.735604195279909E-07</v>
       </c>
     </row>
     <row r="7">
@@ -481,10 +482,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.1176</v>
+        <v>0.2409972299168975</v>
       </c>
       <c r="D7">
-        <v>4.461943622118817E-14</v>
+        <v>0.002122022611563511</v>
       </c>
     </row>
   </sheetData>
@@ -531,10 +532,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.2409946417943777</v>
+        <v>0.2409946417943775</v>
       </c>
       <c r="D2">
-        <v>0.09529596052654776</v>
+        <v>0.09529596052654821</v>
       </c>
     </row>
     <row r="3">
@@ -567,7 +568,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.4016465624792652</v>
+        <v>0.4016465624792653</v>
       </c>
       <c r="D4">
         <v>0.004230060809255809</v>
@@ -585,7 +586,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.5611671771902004</v>
+        <v>0.5611671771902005</v>
       </c>
       <c r="D5">
         <v>2.735352199456642E-05</v>
@@ -603,7 +604,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.2264557778720812</v>
+        <v>0.2264557778720811</v>
       </c>
       <c r="D6">
         <v>0.1176598148571866</v>
@@ -621,7 +622,7 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.3630723600274957</v>
+        <v>0.3630723600274959</v>
       </c>
       <c r="D7">
         <v>0.01034582954412855</v>
@@ -662,12 +663,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>hoval</t>
+          <t>inc</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>inc</t>
+          <t>hoval</t>
         </is>
       </c>
       <c r="C2">
@@ -680,12 +681,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hoval</t>
+          <t>crime</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>crime</t>
+          <t>hoval</t>
         </is>
       </c>
       <c r="C3">
@@ -698,12 +699,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>inc</t>
+          <t>hoval</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>hoval</t>
+          <t>inc</t>
         </is>
       </c>
       <c r="C4">
@@ -716,12 +717,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>inc</t>
+          <t>crime</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>crime</t>
+          <t>inc</t>
         </is>
       </c>
       <c r="C5">
@@ -734,12 +735,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>crime</t>
+          <t>hoval</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>hoval</t>
+          <t>crime</t>
         </is>
       </c>
       <c r="C6">
@@ -752,12 +753,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>crime</t>
+          <t>inc</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>inc</t>
+          <t>crime</t>
         </is>
       </c>
       <c r="C7">
@@ -802,6 +803,146 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>inc</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>hoval</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>1.618478038360967</v>
+      </c>
+      <c r="D2">
+        <v>0.6576551725336324</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>crime</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>hoval</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0.01474868613408025</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>hoval</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>inc</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0.6576551725336324</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>crime</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>inc</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0.002357422376880978</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>hoval</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>crime</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>-0.2739314781716748</v>
+      </c>
+      <c r="D6">
+        <v>0.01474868613408025</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>inc</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>crime</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>-1.597310834084704</v>
+      </c>
+      <c r="D7">
+        <v>0.002357422376880978</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>cause</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>effect</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>cs</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>hoval</t>
         </is>
       </c>

</xml_diff>